<commit_message>
testing production branch change
</commit_message>
<xml_diff>
--- a/user_cart.xlsx
+++ b/user_cart.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,58 +446,6 @@
         <is>
           <t>total_cost</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PER12</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Perfume</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>500</v>
-      </c>
-      <c r="F2" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Pas12</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Pasta</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>100</v>
-      </c>
-      <c r="F3" t="n">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>